<commit_message>
Updated ZWE model - 2025-09-16 22:36
</commit_message>
<xml_diff>
--- a/VerveStacks_ZWE/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ZWE/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZWE\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EDA45D3A-4FD7-4902-BC72-F9E5EDDC41D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C15D294E-8CB2-4113-9E63-FFD922DC9E5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6009,7 +6009,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2A95B00-4BDD-47E2-8C32-483F04B8D551}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63BD4EBE-B335-48B6-BE8F-F16636525433}">
   <dimension ref="B9:N32"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6901,7 +6901,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EA82634-00F0-4182-AB8B-C2C3F848C260}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE8FAE2-D0DE-4D97-BFC2-263B6A6BEBEF}">
   <dimension ref="B9:N30"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7717,7 +7717,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FEC0395-68CA-4037-A389-1369C1281986}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76952536-201F-43A8-B66C-44EEC1E70183}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ZWE model - 2025-09-16 23:45
</commit_message>
<xml_diff>
--- a/VerveStacks_ZWE/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ZWE/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZWE\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C15D294E-8CB2-4113-9E63-FFD922DC9E5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DF0F11A-84D9-4954-AD27-754541A75578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2573" yWindow="2573" windowWidth="21600" windowHeight="12682" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc" sheetId="7" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="339">
   <si>
     <t>~FI_Process</t>
   </si>
@@ -815,9 +815,6 @@
   </si>
   <si>
     <t>solar resource in cluster 22</t>
-  </si>
-  <si>
-    <t>cluster_id</t>
   </si>
   <si>
     <t>comm-out</t>
@@ -6009,11 +6006,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63BD4EBE-B335-48B6-BE8F-F16636525433}">
-  <dimension ref="B9:N32"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{228CC0F7-74C7-4FFE-9724-9431B99186D6}">
+  <dimension ref="B9:M32"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="9" spans="2:14">
+    <row r="9" spans="2:13">
       <c r="B9" t="s">
         <v>163</v>
       </c>
@@ -6021,7 +6018,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="10" spans="2:14">
+    <row r="10" spans="2:13">
       <c r="B10" t="s">
         <v>178</v>
       </c>
@@ -6044,10 +6041,10 @@
         <v>181</v>
       </c>
       <c r="J10" t="s">
+        <v>164</v>
+      </c>
+      <c r="K10" t="s">
         <v>229</v>
-      </c>
-      <c r="K10" t="s">
-        <v>164</v>
       </c>
       <c r="L10" t="s">
         <v>230</v>
@@ -6055,11 +6052,8 @@
       <c r="M10" t="s">
         <v>231</v>
       </c>
-      <c r="N10" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="11" spans="2:14">
+    </row>
+    <row r="11" spans="2:13">
       <c r="B11" t="s">
         <v>182</v>
       </c>
@@ -6081,23 +6075,20 @@
       <c r="H11" t="s">
         <v>186</v>
       </c>
-      <c r="J11">
-        <v>1</v>
+      <c r="J11" t="s">
+        <v>183</v>
       </c>
       <c r="K11" t="s">
-        <v>183</v>
-      </c>
-      <c r="L11" t="s">
-        <v>233</v>
+        <v>232</v>
+      </c>
+      <c r="L11">
+        <v>13.520978908906518</v>
       </c>
       <c r="M11">
-        <v>3.5936526597163057</v>
-      </c>
-      <c r="N11">
-        <v>0.2049312065675559</v>
-      </c>
-    </row>
-    <row r="12" spans="2:14">
+        <v>0.2284487086259582</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13">
       <c r="B12" t="s">
         <v>182</v>
       </c>
@@ -6119,23 +6110,20 @@
       <c r="H12" t="s">
         <v>186</v>
       </c>
-      <c r="J12">
-        <v>2</v>
+      <c r="J12" t="s">
+        <v>187</v>
       </c>
       <c r="K12" t="s">
-        <v>187</v>
-      </c>
-      <c r="L12" t="s">
-        <v>234</v>
+        <v>233</v>
+      </c>
+      <c r="L12">
+        <v>10.791470258613435</v>
       </c>
       <c r="M12">
-        <v>2.9809312249086122</v>
-      </c>
-      <c r="N12">
-        <v>0.21771910320918181</v>
-      </c>
-    </row>
-    <row r="13" spans="2:14">
+        <v>0.2292346780121032</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13">
       <c r="B13" t="s">
         <v>182</v>
       </c>
@@ -6157,23 +6145,20 @@
       <c r="H13" t="s">
         <v>186</v>
       </c>
-      <c r="J13">
-        <v>3</v>
+      <c r="J13" t="s">
+        <v>189</v>
       </c>
       <c r="K13" t="s">
-        <v>189</v>
-      </c>
-      <c r="L13" t="s">
-        <v>235</v>
+        <v>234</v>
+      </c>
+      <c r="L13">
+        <v>2.9809312249086122</v>
       </c>
       <c r="M13">
-        <v>4.9443494406468407</v>
-      </c>
-      <c r="N13">
-        <v>0.21062501811549661</v>
-      </c>
-    </row>
-    <row r="14" spans="2:14">
+        <v>0.21771910320918181</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13">
       <c r="B14" t="s">
         <v>182</v>
       </c>
@@ -6195,23 +6180,20 @@
       <c r="H14" t="s">
         <v>186</v>
       </c>
-      <c r="J14">
-        <v>4</v>
+      <c r="J14" t="s">
+        <v>191</v>
       </c>
       <c r="K14" t="s">
-        <v>191</v>
-      </c>
-      <c r="L14" t="s">
-        <v>236</v>
+        <v>235</v>
+      </c>
+      <c r="L14">
+        <v>5.5402630163144968</v>
       </c>
       <c r="M14">
-        <v>11.912026817262712</v>
-      </c>
-      <c r="N14">
-        <v>0.22879095842898989</v>
-      </c>
-    </row>
-    <row r="15" spans="2:14">
+        <v>0.21022661132739981</v>
+      </c>
+    </row>
+    <row r="15" spans="2:13">
       <c r="B15" t="s">
         <v>182</v>
       </c>
@@ -6233,23 +6215,20 @@
       <c r="H15" t="s">
         <v>186</v>
       </c>
-      <c r="J15">
-        <v>5</v>
+      <c r="J15" t="s">
+        <v>193</v>
       </c>
       <c r="K15" t="s">
-        <v>193</v>
-      </c>
-      <c r="L15" t="s">
-        <v>237</v>
+        <v>236</v>
+      </c>
+      <c r="L15">
+        <v>3.5936526597163057</v>
       </c>
       <c r="M15">
-        <v>6.8789324310860698</v>
-      </c>
-      <c r="N15">
-        <v>0.20420001368463489</v>
-      </c>
-    </row>
-    <row r="16" spans="2:14">
+        <v>0.2049312065675559</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13">
       <c r="B16" t="s">
         <v>182</v>
       </c>
@@ -6271,23 +6250,20 @@
       <c r="H16" t="s">
         <v>186</v>
       </c>
-      <c r="J16">
-        <v>6</v>
+      <c r="J16" t="s">
+        <v>195</v>
       </c>
       <c r="K16" t="s">
-        <v>195</v>
-      </c>
-      <c r="L16" t="s">
-        <v>238</v>
+        <v>237</v>
+      </c>
+      <c r="L16">
+        <v>5.8948902378723158</v>
       </c>
       <c r="M16">
-        <v>13.237580400364452</v>
-      </c>
-      <c r="N16">
-        <v>0.21168170592681981</v>
-      </c>
-    </row>
-    <row r="17" spans="2:14">
+        <v>0.2150350980628645</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13">
       <c r="B17" t="s">
         <v>182</v>
       </c>
@@ -6309,23 +6285,20 @@
       <c r="H17" t="s">
         <v>186</v>
       </c>
-      <c r="J17">
-        <v>7</v>
+      <c r="J17" t="s">
+        <v>197</v>
       </c>
       <c r="K17" t="s">
-        <v>197</v>
-      </c>
-      <c r="L17" t="s">
-        <v>239</v>
+        <v>238</v>
+      </c>
+      <c r="L17">
+        <v>6.8789324310860698</v>
       </c>
       <c r="M17">
-        <v>5.3628765951031694</v>
-      </c>
-      <c r="N17">
-        <v>0.2227680720596969</v>
-      </c>
-    </row>
-    <row r="18" spans="2:14">
+        <v>0.20420001368463489</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13">
       <c r="B18" t="s">
         <v>182</v>
       </c>
@@ -6347,23 +6320,20 @@
       <c r="H18" t="s">
         <v>186</v>
       </c>
-      <c r="J18">
-        <v>8</v>
+      <c r="J18" t="s">
+        <v>199</v>
       </c>
       <c r="K18" t="s">
-        <v>199</v>
-      </c>
-      <c r="L18" t="s">
-        <v>240</v>
+        <v>239</v>
+      </c>
+      <c r="L18">
+        <v>13.237580400364452</v>
       </c>
       <c r="M18">
-        <v>4.9818620713796955</v>
-      </c>
-      <c r="N18">
-        <v>0.2129572805063393</v>
-      </c>
-    </row>
-    <row r="19" spans="2:14">
+        <v>0.21168170592681981</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13">
       <c r="B19" t="s">
         <v>182</v>
       </c>
@@ -6385,23 +6355,20 @@
       <c r="H19" t="s">
         <v>186</v>
       </c>
-      <c r="J19">
-        <v>9</v>
+      <c r="J19" t="s">
+        <v>201</v>
       </c>
       <c r="K19" t="s">
-        <v>201</v>
-      </c>
-      <c r="L19" t="s">
-        <v>241</v>
+        <v>240</v>
+      </c>
+      <c r="L19">
+        <v>1.102581581823173</v>
       </c>
       <c r="M19">
-        <v>3.4211924277552983</v>
-      </c>
-      <c r="N19">
-        <v>0.2302515900737192</v>
-      </c>
-    </row>
-    <row r="20" spans="2:14">
+        <v>0.22461071972716781</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13">
       <c r="B20" t="s">
         <v>182</v>
       </c>
@@ -6423,23 +6390,20 @@
       <c r="H20" t="s">
         <v>186</v>
       </c>
-      <c r="J20">
-        <v>10</v>
+      <c r="J20" t="s">
+        <v>203</v>
       </c>
       <c r="K20" t="s">
-        <v>203</v>
-      </c>
-      <c r="L20" t="s">
-        <v>242</v>
+        <v>241</v>
+      </c>
+      <c r="L20">
+        <v>2.3186108459321253</v>
       </c>
       <c r="M20">
-        <v>5.3751413942157447</v>
-      </c>
-      <c r="N20">
-        <v>0.22464053013276669</v>
-      </c>
-    </row>
-    <row r="21" spans="2:14">
+        <v>0.23293402372163891</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13">
       <c r="B21" t="s">
         <v>182</v>
       </c>
@@ -6461,23 +6425,20 @@
       <c r="H21" t="s">
         <v>186</v>
       </c>
-      <c r="J21">
-        <v>11</v>
+      <c r="J21" t="s">
+        <v>205</v>
       </c>
       <c r="K21" t="s">
-        <v>205</v>
-      </c>
-      <c r="L21" t="s">
-        <v>243</v>
+        <v>242</v>
+      </c>
+      <c r="L21">
+        <v>4.7015231746671615</v>
       </c>
       <c r="M21">
-        <v>6.2591685344698025</v>
-      </c>
-      <c r="N21">
-        <v>0.23215881267948721</v>
-      </c>
-    </row>
-    <row r="22" spans="2:14">
+        <v>0.2334118661248904</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13">
       <c r="B22" t="s">
         <v>182</v>
       </c>
@@ -6499,23 +6460,20 @@
       <c r="H22" t="s">
         <v>186</v>
       </c>
-      <c r="J22">
-        <v>12</v>
+      <c r="J22" t="s">
+        <v>207</v>
       </c>
       <c r="K22" t="s">
-        <v>207</v>
-      </c>
-      <c r="L22" t="s">
-        <v>244</v>
+        <v>243</v>
+      </c>
+      <c r="L22">
+        <v>8.4574615470220227</v>
       </c>
       <c r="M22">
-        <v>4.7494886805227079</v>
-      </c>
-      <c r="N22">
-        <v>0.23697327684511771</v>
-      </c>
-    </row>
-    <row r="23" spans="2:14">
+        <v>0.22655216953553989</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13">
       <c r="B23" t="s">
         <v>182</v>
       </c>
@@ -6537,23 +6495,20 @@
       <c r="H23" t="s">
         <v>186</v>
       </c>
-      <c r="J23">
-        <v>13</v>
+      <c r="J23" t="s">
+        <v>209</v>
       </c>
       <c r="K23" t="s">
-        <v>209</v>
-      </c>
-      <c r="L23" t="s">
-        <v>245</v>
+        <v>244</v>
+      </c>
+      <c r="L23">
+        <v>4.7494886805227079</v>
       </c>
       <c r="M23">
-        <v>10.5181177861111</v>
-      </c>
-      <c r="N23">
-        <v>0.2334001870115136</v>
-      </c>
-    </row>
-    <row r="24" spans="2:14">
+        <v>0.23697327684511771</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13">
       <c r="B24" t="s">
         <v>182</v>
       </c>
@@ -6575,23 +6530,20 @@
       <c r="H24" t="s">
         <v>186</v>
       </c>
-      <c r="J24">
-        <v>14</v>
+      <c r="J24" t="s">
+        <v>211</v>
       </c>
       <c r="K24" t="s">
-        <v>211</v>
-      </c>
-      <c r="L24" t="s">
-        <v>246</v>
+        <v>245</v>
+      </c>
+      <c r="L24">
+        <v>10.5181177861111</v>
       </c>
       <c r="M24">
-        <v>8.7942897522313199</v>
-      </c>
-      <c r="N24">
-        <v>0.2378651747752859</v>
-      </c>
-    </row>
-    <row r="25" spans="2:14">
+        <v>0.2334001870115136</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13">
       <c r="B25" t="s">
         <v>182</v>
       </c>
@@ -6613,23 +6565,20 @@
       <c r="H25" t="s">
         <v>186</v>
       </c>
-      <c r="J25">
-        <v>15</v>
+      <c r="J25" t="s">
+        <v>213</v>
       </c>
       <c r="K25" t="s">
-        <v>213</v>
-      </c>
-      <c r="L25" t="s">
-        <v>247</v>
+        <v>246</v>
+      </c>
+      <c r="L25">
+        <v>6.1074171567218594</v>
       </c>
       <c r="M25">
-        <v>6.1074171567218594</v>
-      </c>
-      <c r="N25">
         <v>0.2355366195227285</v>
       </c>
     </row>
-    <row r="26" spans="2:14">
+    <row r="26" spans="2:13">
       <c r="B26" t="s">
         <v>182</v>
       </c>
@@ -6651,23 +6600,20 @@
       <c r="H26" t="s">
         <v>186</v>
       </c>
-      <c r="J26">
-        <v>16</v>
+      <c r="J26" t="s">
+        <v>215</v>
       </c>
       <c r="K26" t="s">
-        <v>215</v>
-      </c>
-      <c r="L26" t="s">
-        <v>248</v>
+        <v>247</v>
+      </c>
+      <c r="L26">
+        <v>9.7553892592945122</v>
       </c>
       <c r="M26">
-        <v>9.7553892592945122</v>
-      </c>
-      <c r="N26">
         <v>0.23369950307670509</v>
       </c>
     </row>
-    <row r="27" spans="2:14">
+    <row r="27" spans="2:13">
       <c r="B27" t="s">
         <v>182</v>
       </c>
@@ -6689,23 +6635,20 @@
       <c r="H27" t="s">
         <v>186</v>
       </c>
-      <c r="J27">
-        <v>17</v>
+      <c r="J27" t="s">
+        <v>217</v>
       </c>
       <c r="K27" t="s">
-        <v>217</v>
-      </c>
-      <c r="L27" t="s">
-        <v>249</v>
+        <v>248</v>
+      </c>
+      <c r="L27">
+        <v>3.4589805482800817</v>
       </c>
       <c r="M27">
-        <v>13.570796249372853</v>
-      </c>
-      <c r="N27">
-        <v>0.23741901532562479</v>
-      </c>
-    </row>
-    <row r="28" spans="2:14">
+        <v>0.23753765256535511</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13">
       <c r="B28" t="s">
         <v>182</v>
       </c>
@@ -6727,23 +6670,20 @@
       <c r="H28" t="s">
         <v>186</v>
       </c>
-      <c r="J28">
-        <v>18</v>
+      <c r="J28" t="s">
+        <v>219</v>
       </c>
       <c r="K28" t="s">
-        <v>219</v>
-      </c>
-      <c r="L28" t="s">
-        <v>250</v>
+        <v>249</v>
+      </c>
+      <c r="L28">
+        <v>8.7942897522313199</v>
       </c>
       <c r="M28">
-        <v>3.4589805482800817</v>
-      </c>
-      <c r="N28">
-        <v>0.23753765256535511</v>
-      </c>
-    </row>
-    <row r="29" spans="2:14">
+        <v>0.2378651747752859</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13">
       <c r="B29" t="s">
         <v>182</v>
       </c>
@@ -6765,23 +6705,20 @@
       <c r="H29" t="s">
         <v>186</v>
       </c>
-      <c r="J29">
-        <v>19</v>
+      <c r="J29" t="s">
+        <v>221</v>
       </c>
       <c r="K29" t="s">
-        <v>221</v>
-      </c>
-      <c r="L29" t="s">
-        <v>251</v>
+        <v>250</v>
+      </c>
+      <c r="L29">
+        <v>13.570796249372853</v>
       </c>
       <c r="M29">
-        <v>10.071162290317991</v>
-      </c>
-      <c r="N29">
-        <v>0.23089996421623421</v>
-      </c>
-    </row>
-    <row r="30" spans="2:14">
+        <v>0.23741901532562479</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13">
       <c r="B30" t="s">
         <v>182</v>
       </c>
@@ -6803,23 +6740,20 @@
       <c r="H30" t="s">
         <v>186</v>
       </c>
-      <c r="J30">
-        <v>20</v>
+      <c r="J30" t="s">
+        <v>223</v>
       </c>
       <c r="K30" t="s">
-        <v>223</v>
-      </c>
-      <c r="L30" t="s">
-        <v>252</v>
+        <v>251</v>
+      </c>
+      <c r="L30">
+        <v>16.487357011033904</v>
       </c>
       <c r="M30">
-        <v>16.487357011033904</v>
-      </c>
-      <c r="N30">
         <v>0.23465680723655979</v>
       </c>
     </row>
-    <row r="31" spans="2:14">
+    <row r="31" spans="2:13">
       <c r="B31" t="s">
         <v>182</v>
       </c>
@@ -6841,23 +6775,20 @@
       <c r="H31" t="s">
         <v>186</v>
       </c>
-      <c r="J31">
-        <v>21</v>
+      <c r="J31" t="s">
+        <v>225</v>
       </c>
       <c r="K31" t="s">
-        <v>225</v>
-      </c>
-      <c r="L31" t="s">
-        <v>253</v>
+        <v>252</v>
+      </c>
+      <c r="L31">
+        <v>6.2049288245335807</v>
       </c>
       <c r="M31">
-        <v>6.2049288245335807</v>
-      </c>
-      <c r="N31">
         <v>0.23840447108523369</v>
       </c>
     </row>
-    <row r="32" spans="2:14">
+    <row r="32" spans="2:13">
       <c r="B32" t="s">
         <v>182</v>
       </c>
@@ -6879,19 +6810,16 @@
       <c r="H32" t="s">
         <v>186</v>
       </c>
-      <c r="J32">
-        <v>22</v>
+      <c r="J32" t="s">
+        <v>227</v>
       </c>
       <c r="K32" t="s">
-        <v>227</v>
-      </c>
-      <c r="L32" t="s">
-        <v>254</v>
+        <v>253</v>
+      </c>
+      <c r="L32">
+        <v>11.987124717844024</v>
       </c>
       <c r="M32">
-        <v>11.987124717844024</v>
-      </c>
-      <c r="N32">
         <v>0.23615841714686039</v>
       </c>
     </row>
@@ -6901,11 +6829,11 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE8FAE2-D0DE-4D97-BFC2-263B6A6BEBEF}">
-  <dimension ref="B9:N30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF0BFFFF-66D7-4C40-A55E-3E9652F22240}">
+  <dimension ref="B9:M30"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="9" spans="2:14">
+    <row r="9" spans="2:13">
       <c r="B9" t="s">
         <v>163</v>
       </c>
@@ -6913,7 +6841,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="10" spans="2:14">
+    <row r="10" spans="2:13">
       <c r="B10" t="s">
         <v>178</v>
       </c>
@@ -6936,10 +6864,10 @@
         <v>181</v>
       </c>
       <c r="J10" t="s">
+        <v>164</v>
+      </c>
+      <c r="K10" t="s">
         <v>229</v>
-      </c>
-      <c r="K10" t="s">
-        <v>164</v>
       </c>
       <c r="L10" t="s">
         <v>230</v>
@@ -6947,19 +6875,16 @@
       <c r="M10" t="s">
         <v>231</v>
       </c>
-      <c r="N10" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="11" spans="2:14">
+    </row>
+    <row r="11" spans="2:13">
       <c r="B11" t="s">
         <v>182</v>
       </c>
       <c r="C11" t="s">
+        <v>254</v>
+      </c>
+      <c r="D11" t="s">
         <v>255</v>
-      </c>
-      <c r="D11" t="s">
-        <v>256</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -6973,31 +6898,28 @@
       <c r="H11" t="s">
         <v>186</v>
       </c>
-      <c r="J11">
-        <v>1</v>
+      <c r="J11" t="s">
+        <v>254</v>
       </c>
       <c r="K11" t="s">
-        <v>255</v>
-      </c>
-      <c r="L11" t="s">
-        <v>295</v>
+        <v>294</v>
+      </c>
+      <c r="L11">
+        <v>3.1593836917186042</v>
       </c>
       <c r="M11">
-        <v>3.1593836917186042</v>
-      </c>
-      <c r="N11">
         <v>0.2177626206778491</v>
       </c>
     </row>
-    <row r="12" spans="2:14">
+    <row r="12" spans="2:13">
       <c r="B12" t="s">
         <v>182</v>
       </c>
       <c r="C12" t="s">
+        <v>256</v>
+      </c>
+      <c r="D12" t="s">
         <v>257</v>
-      </c>
-      <c r="D12" t="s">
-        <v>258</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -7011,31 +6933,28 @@
       <c r="H12" t="s">
         <v>186</v>
       </c>
-      <c r="J12">
-        <v>2</v>
+      <c r="J12" t="s">
+        <v>256</v>
       </c>
       <c r="K12" t="s">
-        <v>257</v>
-      </c>
-      <c r="L12" t="s">
-        <v>296</v>
+        <v>295</v>
+      </c>
+      <c r="L12">
+        <v>8.6193167216199029</v>
       </c>
       <c r="M12">
-        <v>8.6193167216199029</v>
-      </c>
-      <c r="N12">
         <v>0.25138985782671908</v>
       </c>
     </row>
-    <row r="13" spans="2:14">
+    <row r="13" spans="2:13">
       <c r="B13" t="s">
         <v>182</v>
       </c>
       <c r="C13" t="s">
+        <v>258</v>
+      </c>
+      <c r="D13" t="s">
         <v>259</v>
-      </c>
-      <c r="D13" t="s">
-        <v>260</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -7049,31 +6968,28 @@
       <c r="H13" t="s">
         <v>186</v>
       </c>
-      <c r="J13">
-        <v>3</v>
+      <c r="J13" t="s">
+        <v>258</v>
       </c>
       <c r="K13" t="s">
-        <v>259</v>
-      </c>
-      <c r="L13" t="s">
-        <v>297</v>
+        <v>296</v>
+      </c>
+      <c r="L13">
+        <v>2.9791450296274822</v>
       </c>
       <c r="M13">
-        <v>2.9791450296274822</v>
-      </c>
-      <c r="N13">
         <v>0.20563227244996729</v>
       </c>
     </row>
-    <row r="14" spans="2:14">
+    <row r="14" spans="2:13">
       <c r="B14" t="s">
         <v>182</v>
       </c>
       <c r="C14" t="s">
+        <v>260</v>
+      </c>
+      <c r="D14" t="s">
         <v>261</v>
-      </c>
-      <c r="D14" t="s">
-        <v>262</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -7087,31 +7003,28 @@
       <c r="H14" t="s">
         <v>186</v>
       </c>
-      <c r="J14">
-        <v>4</v>
+      <c r="J14" t="s">
+        <v>260</v>
       </c>
       <c r="K14" t="s">
-        <v>261</v>
-      </c>
-      <c r="L14" t="s">
-        <v>298</v>
+        <v>297</v>
+      </c>
+      <c r="L14">
+        <v>0.14554397292815968</v>
       </c>
       <c r="M14">
-        <v>0.14554397292815968</v>
-      </c>
-      <c r="N14">
         <v>0.1083895443562508</v>
       </c>
     </row>
-    <row r="15" spans="2:14">
+    <row r="15" spans="2:13">
       <c r="B15" t="s">
         <v>182</v>
       </c>
       <c r="C15" t="s">
+        <v>262</v>
+      </c>
+      <c r="D15" t="s">
         <v>263</v>
-      </c>
-      <c r="D15" t="s">
-        <v>264</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -7125,31 +7038,28 @@
       <c r="H15" t="s">
         <v>186</v>
       </c>
-      <c r="J15">
-        <v>5</v>
+      <c r="J15" t="s">
+        <v>262</v>
       </c>
       <c r="K15" t="s">
-        <v>263</v>
-      </c>
-      <c r="L15" t="s">
-        <v>299</v>
+        <v>298</v>
+      </c>
+      <c r="L15">
+        <v>0.92998773115040478</v>
       </c>
       <c r="M15">
-        <v>0.92998773115040478</v>
-      </c>
-      <c r="N15">
         <v>0.1718244595248172</v>
       </c>
     </row>
-    <row r="16" spans="2:14">
+    <row r="16" spans="2:13">
       <c r="B16" t="s">
         <v>182</v>
       </c>
       <c r="C16" t="s">
+        <v>264</v>
+      </c>
+      <c r="D16" t="s">
         <v>265</v>
-      </c>
-      <c r="D16" t="s">
-        <v>266</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -7163,31 +7073,28 @@
       <c r="H16" t="s">
         <v>186</v>
       </c>
-      <c r="J16">
-        <v>6</v>
+      <c r="J16" t="s">
+        <v>264</v>
       </c>
       <c r="K16" t="s">
-        <v>265</v>
-      </c>
-      <c r="L16" t="s">
-        <v>300</v>
+        <v>299</v>
+      </c>
+      <c r="L16">
+        <v>11.716439286103554</v>
       </c>
       <c r="M16">
-        <v>11.716439286103554</v>
-      </c>
-      <c r="N16">
         <v>0.29053106041645349</v>
       </c>
     </row>
-    <row r="17" spans="2:14">
+    <row r="17" spans="2:13">
       <c r="B17" t="s">
         <v>182</v>
       </c>
       <c r="C17" t="s">
+        <v>266</v>
+      </c>
+      <c r="D17" t="s">
         <v>267</v>
-      </c>
-      <c r="D17" t="s">
-        <v>268</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -7201,31 +7108,28 @@
       <c r="H17" t="s">
         <v>186</v>
       </c>
-      <c r="J17">
-        <v>7</v>
+      <c r="J17" t="s">
+        <v>266</v>
       </c>
       <c r="K17" t="s">
-        <v>267</v>
-      </c>
-      <c r="L17" t="s">
-        <v>301</v>
+        <v>300</v>
+      </c>
+      <c r="L17">
+        <v>9.3471093911156089</v>
       </c>
       <c r="M17">
-        <v>9.3471093911156089</v>
-      </c>
-      <c r="N17">
         <v>0.24982751695624381</v>
       </c>
     </row>
-    <row r="18" spans="2:14">
+    <row r="18" spans="2:13">
       <c r="B18" t="s">
         <v>182</v>
       </c>
       <c r="C18" t="s">
+        <v>268</v>
+      </c>
+      <c r="D18" t="s">
         <v>269</v>
-      </c>
-      <c r="D18" t="s">
-        <v>270</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -7239,31 +7143,28 @@
       <c r="H18" t="s">
         <v>186</v>
       </c>
-      <c r="J18">
-        <v>8</v>
+      <c r="J18" t="s">
+        <v>268</v>
       </c>
       <c r="K18" t="s">
-        <v>269</v>
-      </c>
-      <c r="L18" t="s">
-        <v>302</v>
+        <v>301</v>
+      </c>
+      <c r="L18">
+        <v>1.0606909440829149</v>
       </c>
       <c r="M18">
-        <v>1.0606909440829149</v>
-      </c>
-      <c r="N18">
         <v>0.17223836830704731</v>
       </c>
     </row>
-    <row r="19" spans="2:14">
+    <row r="19" spans="2:13">
       <c r="B19" t="s">
         <v>182</v>
       </c>
       <c r="C19" t="s">
+        <v>270</v>
+      </c>
+      <c r="D19" t="s">
         <v>271</v>
-      </c>
-      <c r="D19" t="s">
-        <v>272</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -7277,31 +7178,28 @@
       <c r="H19" t="s">
         <v>186</v>
       </c>
-      <c r="J19">
-        <v>9</v>
+      <c r="J19" t="s">
+        <v>270</v>
       </c>
       <c r="K19" t="s">
-        <v>271</v>
-      </c>
-      <c r="L19" t="s">
-        <v>303</v>
+        <v>302</v>
+      </c>
+      <c r="L19">
+        <v>2.6885012049255272</v>
       </c>
       <c r="M19">
-        <v>2.6885012049255272</v>
-      </c>
-      <c r="N19">
         <v>0.1865630817679394</v>
       </c>
     </row>
-    <row r="20" spans="2:14">
+    <row r="20" spans="2:13">
       <c r="B20" t="s">
         <v>182</v>
       </c>
       <c r="C20" t="s">
+        <v>272</v>
+      </c>
+      <c r="D20" t="s">
         <v>273</v>
-      </c>
-      <c r="D20" t="s">
-        <v>274</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -7315,31 +7213,28 @@
       <c r="H20" t="s">
         <v>186</v>
       </c>
-      <c r="J20">
-        <v>10</v>
+      <c r="J20" t="s">
+        <v>272</v>
       </c>
       <c r="K20" t="s">
-        <v>273</v>
-      </c>
-      <c r="L20" t="s">
-        <v>304</v>
+        <v>303</v>
+      </c>
+      <c r="L20">
+        <v>2.4179169789740365</v>
       </c>
       <c r="M20">
-        <v>2.4179169789740365</v>
-      </c>
-      <c r="N20">
         <v>0.17538615389463769</v>
       </c>
     </row>
-    <row r="21" spans="2:14">
+    <row r="21" spans="2:13">
       <c r="B21" t="s">
         <v>182</v>
       </c>
       <c r="C21" t="s">
+        <v>274</v>
+      </c>
+      <c r="D21" t="s">
         <v>275</v>
-      </c>
-      <c r="D21" t="s">
-        <v>276</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -7353,31 +7248,28 @@
       <c r="H21" t="s">
         <v>186</v>
       </c>
-      <c r="J21">
-        <v>11</v>
+      <c r="J21" t="s">
+        <v>274</v>
       </c>
       <c r="K21" t="s">
-        <v>275</v>
-      </c>
-      <c r="L21" t="s">
-        <v>305</v>
+        <v>304</v>
+      </c>
+      <c r="L21">
+        <v>0.52269793829938715</v>
       </c>
       <c r="M21">
-        <v>0.52269793829938715</v>
-      </c>
-      <c r="N21">
         <v>0.1595021667582546</v>
       </c>
     </row>
-    <row r="22" spans="2:14">
+    <row r="22" spans="2:13">
       <c r="B22" t="s">
         <v>182</v>
       </c>
       <c r="C22" t="s">
+        <v>276</v>
+      </c>
+      <c r="D22" t="s">
         <v>277</v>
-      </c>
-      <c r="D22" t="s">
-        <v>278</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -7391,31 +7283,28 @@
       <c r="H22" t="s">
         <v>186</v>
       </c>
-      <c r="J22">
-        <v>12</v>
+      <c r="J22" t="s">
+        <v>276</v>
       </c>
       <c r="K22" t="s">
-        <v>277</v>
-      </c>
-      <c r="L22" t="s">
-        <v>306</v>
+        <v>305</v>
+      </c>
+      <c r="L22">
+        <v>5.4958744424097663</v>
       </c>
       <c r="M22">
-        <v>5.4958744424097663</v>
-      </c>
-      <c r="N22">
         <v>0.21867101838220279</v>
       </c>
     </row>
-    <row r="23" spans="2:14">
+    <row r="23" spans="2:13">
       <c r="B23" t="s">
         <v>182</v>
       </c>
       <c r="C23" t="s">
+        <v>278</v>
+      </c>
+      <c r="D23" t="s">
         <v>279</v>
-      </c>
-      <c r="D23" t="s">
-        <v>280</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -7429,31 +7318,28 @@
       <c r="H23" t="s">
         <v>186</v>
       </c>
-      <c r="J23">
-        <v>13</v>
+      <c r="J23" t="s">
+        <v>278</v>
       </c>
       <c r="K23" t="s">
-        <v>279</v>
-      </c>
-      <c r="L23" t="s">
-        <v>307</v>
+        <v>306</v>
+      </c>
+      <c r="L23">
+        <v>2.6982123914524814</v>
       </c>
       <c r="M23">
-        <v>2.6982123914524814</v>
-      </c>
-      <c r="N23">
         <v>0.2244395064502086</v>
       </c>
     </row>
-    <row r="24" spans="2:14">
+    <row r="24" spans="2:13">
       <c r="B24" t="s">
         <v>182</v>
       </c>
       <c r="C24" t="s">
+        <v>280</v>
+      </c>
+      <c r="D24" t="s">
         <v>281</v>
-      </c>
-      <c r="D24" t="s">
-        <v>282</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -7467,31 +7353,28 @@
       <c r="H24" t="s">
         <v>186</v>
       </c>
-      <c r="J24">
-        <v>14</v>
+      <c r="J24" t="s">
+        <v>280</v>
       </c>
       <c r="K24" t="s">
-        <v>281</v>
-      </c>
-      <c r="L24" t="s">
-        <v>308</v>
+        <v>307</v>
+      </c>
+      <c r="L24">
+        <v>0.4880329602108382</v>
       </c>
       <c r="M24">
-        <v>0.4880329602108382</v>
-      </c>
-      <c r="N24">
         <v>0.17197221103856081</v>
       </c>
     </row>
-    <row r="25" spans="2:14">
+    <row r="25" spans="2:13">
       <c r="B25" t="s">
         <v>182</v>
       </c>
       <c r="C25" t="s">
+        <v>282</v>
+      </c>
+      <c r="D25" t="s">
         <v>283</v>
-      </c>
-      <c r="D25" t="s">
-        <v>284</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -7505,31 +7388,28 @@
       <c r="H25" t="s">
         <v>186</v>
       </c>
-      <c r="J25">
-        <v>15</v>
+      <c r="J25" t="s">
+        <v>282</v>
       </c>
       <c r="K25" t="s">
-        <v>283</v>
-      </c>
-      <c r="L25" t="s">
-        <v>309</v>
+        <v>308</v>
+      </c>
+      <c r="L25">
+        <v>0.39527318593380312</v>
       </c>
       <c r="M25">
-        <v>0.39527318593380312</v>
-      </c>
-      <c r="N25">
         <v>0.14281288676747231</v>
       </c>
     </row>
-    <row r="26" spans="2:14">
+    <row r="26" spans="2:13">
       <c r="B26" t="s">
         <v>182</v>
       </c>
       <c r="C26" t="s">
+        <v>284</v>
+      </c>
+      <c r="D26" t="s">
         <v>285</v>
-      </c>
-      <c r="D26" t="s">
-        <v>286</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -7543,31 +7423,28 @@
       <c r="H26" t="s">
         <v>186</v>
       </c>
-      <c r="J26">
-        <v>16</v>
+      <c r="J26" t="s">
+        <v>284</v>
       </c>
       <c r="K26" t="s">
-        <v>285</v>
-      </c>
-      <c r="L26" t="s">
-        <v>310</v>
+        <v>309</v>
+      </c>
+      <c r="L26">
+        <v>0.34302511151375481</v>
       </c>
       <c r="M26">
-        <v>0.34302511151375481</v>
-      </c>
-      <c r="N26">
         <v>0.1574991090533672</v>
       </c>
     </row>
-    <row r="27" spans="2:14">
+    <row r="27" spans="2:13">
       <c r="B27" t="s">
         <v>182</v>
       </c>
       <c r="C27" t="s">
+        <v>286</v>
+      </c>
+      <c r="D27" t="s">
         <v>287</v>
-      </c>
-      <c r="D27" t="s">
-        <v>288</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -7581,31 +7458,28 @@
       <c r="H27" t="s">
         <v>186</v>
       </c>
-      <c r="J27">
-        <v>17</v>
+      <c r="J27" t="s">
+        <v>286</v>
       </c>
       <c r="K27" t="s">
-        <v>287</v>
-      </c>
-      <c r="L27" t="s">
-        <v>311</v>
+        <v>310</v>
+      </c>
+      <c r="L27">
+        <v>8.7533867381102248E-2</v>
       </c>
       <c r="M27">
-        <v>8.7533867381102248E-2</v>
-      </c>
-      <c r="N27">
         <v>9.5260017605740294E-2</v>
       </c>
     </row>
-    <row r="28" spans="2:14">
+    <row r="28" spans="2:13">
       <c r="B28" t="s">
         <v>182</v>
       </c>
       <c r="C28" t="s">
+        <v>288</v>
+      </c>
+      <c r="D28" t="s">
         <v>289</v>
-      </c>
-      <c r="D28" t="s">
-        <v>290</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -7619,31 +7493,28 @@
       <c r="H28" t="s">
         <v>186</v>
       </c>
-      <c r="J28">
-        <v>18</v>
+      <c r="J28" t="s">
+        <v>288</v>
       </c>
       <c r="K28" t="s">
-        <v>289</v>
-      </c>
-      <c r="L28" t="s">
-        <v>312</v>
+        <v>311</v>
+      </c>
+      <c r="L28">
+        <v>0.55790763236243379</v>
       </c>
       <c r="M28">
-        <v>0.55790763236243379</v>
-      </c>
-      <c r="N28">
         <v>0.11947974039484539</v>
       </c>
     </row>
-    <row r="29" spans="2:14">
+    <row r="29" spans="2:13">
       <c r="B29" t="s">
         <v>182</v>
       </c>
       <c r="C29" t="s">
+        <v>290</v>
+      </c>
+      <c r="D29" t="s">
         <v>291</v>
-      </c>
-      <c r="D29" t="s">
-        <v>292</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -7657,31 +7528,28 @@
       <c r="H29" t="s">
         <v>186</v>
       </c>
-      <c r="J29">
-        <v>19</v>
+      <c r="J29" t="s">
+        <v>290</v>
       </c>
       <c r="K29" t="s">
-        <v>291</v>
-      </c>
-      <c r="L29" t="s">
-        <v>313</v>
+        <v>312</v>
+      </c>
+      <c r="L29">
+        <v>2.7877492402512845</v>
       </c>
       <c r="M29">
-        <v>2.7877492402512845</v>
-      </c>
-      <c r="N29">
         <v>0.16543161018197289</v>
       </c>
     </row>
-    <row r="30" spans="2:14">
+    <row r="30" spans="2:13">
       <c r="B30" t="s">
         <v>182</v>
       </c>
       <c r="C30" t="s">
+        <v>292</v>
+      </c>
+      <c r="D30" t="s">
         <v>293</v>
-      </c>
-      <c r="D30" t="s">
-        <v>294</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -7695,19 +7563,16 @@
       <c r="H30" t="s">
         <v>186</v>
       </c>
-      <c r="J30">
-        <v>20</v>
+      <c r="J30" t="s">
+        <v>292</v>
       </c>
       <c r="K30" t="s">
-        <v>293</v>
-      </c>
-      <c r="L30" t="s">
-        <v>314</v>
+        <v>313</v>
+      </c>
+      <c r="L30">
+        <v>0.91008235495035117</v>
       </c>
       <c r="M30">
-        <v>0.91008235495035117</v>
-      </c>
-      <c r="N30">
         <v>0.1552446068672137</v>
       </c>
     </row>
@@ -7717,7 +7582,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76952536-201F-43A8-B66C-44EEC1E70183}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B8F1400-49D2-4C36-8EB2-A47B5462D084}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7734,10 +7599,10 @@
         <v>164</v>
       </c>
       <c r="C10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E10">
         <v>2023</v>
@@ -7775,7 +7640,7 @@
     </row>
     <row r="11" spans="2:16">
       <c r="B11" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C11" t="s">
         <v>31</v>
@@ -7799,7 +7664,7 @@
         <v>182</v>
       </c>
       <c r="K11" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M11" t="s">
         <v>10</v>
@@ -7808,15 +7673,15 @@
         <v>21</v>
       </c>
       <c r="O11" t="s">
+        <v>337</v>
+      </c>
+      <c r="P11" t="s">
         <v>338</v>
-      </c>
-      <c r="P11" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="12" spans="2:16">
       <c r="B12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C12" t="s">
         <v>31</v>
@@ -7834,13 +7699,13 @@
         <v>0.5</v>
       </c>
       <c r="H12" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="J12" t="s">
         <v>182</v>
       </c>
       <c r="K12" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="M12" t="s">
         <v>10</v>
@@ -7849,15 +7714,15 @@
         <v>21</v>
       </c>
       <c r="O12" t="s">
+        <v>337</v>
+      </c>
+      <c r="P12" t="s">
         <v>338</v>
-      </c>
-      <c r="P12" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="13" spans="2:16">
       <c r="B13" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C13" t="s">
         <v>31</v>
@@ -7875,13 +7740,13 @@
         <v>4400</v>
       </c>
       <c r="H13" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J13" t="s">
         <v>182</v>
       </c>
       <c r="K13" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="M13" t="s">
         <v>10</v>
@@ -7890,15 +7755,15 @@
         <v>21</v>
       </c>
       <c r="O13" t="s">
+        <v>337</v>
+      </c>
+      <c r="P13" t="s">
         <v>338</v>
-      </c>
-      <c r="P13" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="14" spans="2:16">
       <c r="B14" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C14" t="s">
         <v>31</v>
@@ -7916,13 +7781,13 @@
         <v>155</v>
       </c>
       <c r="H14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J14" t="s">
         <v>182</v>
       </c>
       <c r="K14" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="M14" t="s">
         <v>10</v>
@@ -7931,15 +7796,15 @@
         <v>21</v>
       </c>
       <c r="O14" t="s">
+        <v>337</v>
+      </c>
+      <c r="P14" t="s">
         <v>338</v>
-      </c>
-      <c r="P14" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="15" spans="2:16">
       <c r="B15" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C15" t="s">
         <v>31</v>
@@ -7957,13 +7822,13 @@
         <v>3</v>
       </c>
       <c r="H15" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J15" t="s">
         <v>182</v>
       </c>
       <c r="K15" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="M15" t="s">
         <v>10</v>
@@ -7972,15 +7837,15 @@
         <v>21</v>
       </c>
       <c r="O15" t="s">
+        <v>337</v>
+      </c>
+      <c r="P15" t="s">
         <v>338</v>
-      </c>
-      <c r="P15" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="16" spans="2:16">
       <c r="B16" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C16" t="s">
         <v>31</v>
@@ -8004,7 +7869,7 @@
         <v>182</v>
       </c>
       <c r="K16" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="M16" t="s">
         <v>10</v>
@@ -8013,15 +7878,15 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
+        <v>337</v>
+      </c>
+      <c r="P16" t="s">
         <v>338</v>
-      </c>
-      <c r="P16" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="17" spans="2:16">
       <c r="B17" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C17" t="s">
         <v>31</v>
@@ -8039,13 +7904,13 @@
         <v>0.5</v>
       </c>
       <c r="H17" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="J17" t="s">
         <v>182</v>
       </c>
       <c r="K17" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M17" t="s">
         <v>10</v>
@@ -8054,15 +7919,15 @@
         <v>21</v>
       </c>
       <c r="O17" t="s">
+        <v>337</v>
+      </c>
+      <c r="P17" t="s">
         <v>338</v>
-      </c>
-      <c r="P17" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="18" spans="2:16">
       <c r="B18" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C18" t="s">
         <v>31</v>
@@ -8080,13 +7945,13 @@
         <v>2050</v>
       </c>
       <c r="H18" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J18" t="s">
         <v>182</v>
       </c>
       <c r="K18" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="M18" t="s">
         <v>10</v>
@@ -8095,15 +7960,15 @@
         <v>21</v>
       </c>
       <c r="O18" t="s">
+        <v>337</v>
+      </c>
+      <c r="P18" t="s">
         <v>338</v>
-      </c>
-      <c r="P18" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="19" spans="2:16">
       <c r="B19" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C19" t="s">
         <v>31</v>
@@ -8121,13 +7986,13 @@
         <v>70</v>
       </c>
       <c r="H19" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J19" t="s">
         <v>182</v>
       </c>
       <c r="K19" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="M19" t="s">
         <v>10</v>
@@ -8136,15 +8001,15 @@
         <v>21</v>
       </c>
       <c r="O19" t="s">
+        <v>337</v>
+      </c>
+      <c r="P19" t="s">
         <v>338</v>
-      </c>
-      <c r="P19" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="20" spans="2:16">
       <c r="B20" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C20" t="s">
         <v>31</v>
@@ -8162,13 +8027,13 @@
         <v>3</v>
       </c>
       <c r="H20" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J20" t="s">
         <v>182</v>
       </c>
       <c r="K20" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="M20" t="s">
         <v>10</v>
@@ -8177,15 +8042,15 @@
         <v>21</v>
       </c>
       <c r="O20" t="s">
+        <v>337</v>
+      </c>
+      <c r="P20" t="s">
         <v>338</v>
-      </c>
-      <c r="P20" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="21" spans="2:16">
       <c r="B21" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C21" t="s">
         <v>33</v>
@@ -8209,7 +8074,7 @@
         <v>182</v>
       </c>
       <c r="K21" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="M21" t="s">
         <v>10</v>
@@ -8218,15 +8083,15 @@
         <v>21</v>
       </c>
       <c r="O21" t="s">
+        <v>337</v>
+      </c>
+      <c r="P21" t="s">
         <v>338</v>
-      </c>
-      <c r="P21" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="22" spans="2:16">
       <c r="B22" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C22" t="s">
         <v>33</v>
@@ -8244,13 +8109,13 @@
         <v>700</v>
       </c>
       <c r="H22" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J22" t="s">
         <v>182</v>
       </c>
       <c r="K22" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="M22" t="s">
         <v>10</v>
@@ -8259,15 +8124,15 @@
         <v>21</v>
       </c>
       <c r="O22" t="s">
+        <v>337</v>
+      </c>
+      <c r="P22" t="s">
         <v>338</v>
-      </c>
-      <c r="P22" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="23" spans="2:16">
       <c r="B23" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C23" t="s">
         <v>33</v>
@@ -8285,13 +8150,13 @@
         <v>25</v>
       </c>
       <c r="H23" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J23" t="s">
         <v>182</v>
       </c>
       <c r="K23" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="M23" t="s">
         <v>10</v>
@@ -8300,15 +8165,15 @@
         <v>21</v>
       </c>
       <c r="O23" t="s">
+        <v>337</v>
+      </c>
+      <c r="P23" t="s">
         <v>338</v>
-      </c>
-      <c r="P23" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="24" spans="2:16">
       <c r="B24" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C24" t="s">
         <v>33</v>
@@ -8332,7 +8197,7 @@
         <v>182</v>
       </c>
       <c r="K24" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="M24" t="s">
         <v>10</v>
@@ -8341,15 +8206,15 @@
         <v>21</v>
       </c>
       <c r="O24" t="s">
+        <v>337</v>
+      </c>
+      <c r="P24" t="s">
         <v>338</v>
-      </c>
-      <c r="P24" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="25" spans="2:16">
       <c r="B25" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C25" t="s">
         <v>33</v>
@@ -8367,13 +8232,13 @@
         <v>1850</v>
       </c>
       <c r="H25" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J25" t="s">
         <v>182</v>
       </c>
       <c r="K25" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="M25" t="s">
         <v>10</v>
@@ -8382,15 +8247,15 @@
         <v>21</v>
       </c>
       <c r="O25" t="s">
+        <v>337</v>
+      </c>
+      <c r="P25" t="s">
         <v>338</v>
-      </c>
-      <c r="P25" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="26" spans="2:16">
       <c r="B26" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C26" t="s">
         <v>33</v>
@@ -8408,13 +8273,13 @@
         <v>65</v>
       </c>
       <c r="H26" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J26" t="s">
         <v>182</v>
       </c>
       <c r="K26" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="M26" t="s">
         <v>10</v>
@@ -8423,15 +8288,15 @@
         <v>21</v>
       </c>
       <c r="O26" t="s">
+        <v>337</v>
+      </c>
+      <c r="P26" t="s">
         <v>338</v>
-      </c>
-      <c r="P26" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="27" spans="2:16">
       <c r="B27" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C27" t="s">
         <v>32</v>
@@ -8455,7 +8320,7 @@
         <v>182</v>
       </c>
       <c r="K27" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="M27" t="s">
         <v>10</v>
@@ -8464,15 +8329,15 @@
         <v>21</v>
       </c>
       <c r="O27" t="s">
+        <v>337</v>
+      </c>
+      <c r="P27" t="s">
         <v>338</v>
-      </c>
-      <c r="P27" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="28" spans="2:16">
       <c r="B28" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C28" t="s">
         <v>32</v>
@@ -8490,12 +8355,12 @@
         <v>3550</v>
       </c>
       <c r="H28" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="29" spans="2:16">
       <c r="B29" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C29" t="s">
         <v>32</v>
@@ -8513,12 +8378,12 @@
         <v>135</v>
       </c>
       <c r="H29" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="30" spans="2:16">
       <c r="B30" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C30" t="s">
         <v>33</v>
@@ -8541,7 +8406,7 @@
     </row>
     <row r="31" spans="2:16">
       <c r="B31" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C31" t="s">
         <v>33</v>
@@ -8559,12 +8424,12 @@
         <v>400</v>
       </c>
       <c r="H31" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="32" spans="2:16">
       <c r="B32" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C32" t="s">
         <v>33</v>
@@ -8582,12 +8447,12 @@
         <v>20</v>
       </c>
       <c r="H32" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="33" spans="2:8">
       <c r="B33" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C33" t="s">
         <v>28</v>
@@ -8610,7 +8475,7 @@
     </row>
     <row r="34" spans="2:8">
       <c r="B34" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C34" t="s">
         <v>28</v>
@@ -8628,12 +8493,12 @@
         <v>0.5</v>
       </c>
       <c r="H34" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="35" spans="2:8">
       <c r="B35" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C35" t="s">
         <v>28</v>
@@ -8651,12 +8516,12 @@
         <v>2100</v>
       </c>
       <c r="H35" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="36" spans="2:8">
       <c r="B36" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C36" t="s">
         <v>28</v>
@@ -8674,12 +8539,12 @@
         <v>50</v>
       </c>
       <c r="H36" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="37" spans="2:8">
       <c r="B37" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C37" t="s">
         <v>28</v>
@@ -8697,12 +8562,12 @@
         <v>4</v>
       </c>
       <c r="H37" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="38" spans="2:8">
       <c r="B38" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C38" t="s">
         <v>33</v>
@@ -8725,7 +8590,7 @@
     </row>
     <row r="39" spans="2:8">
       <c r="B39" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C39" t="s">
         <v>33</v>
@@ -8743,12 +8608,12 @@
         <v>2100</v>
       </c>
       <c r="H39" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="40" spans="2:8">
       <c r="B40" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C40" t="s">
         <v>33</v>
@@ -8766,12 +8631,12 @@
         <v>85</v>
       </c>
       <c r="H40" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="41" spans="2:8">
       <c r="B41" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C41" t="s">
         <v>32</v>
@@ -8794,7 +8659,7 @@
     </row>
     <row r="42" spans="2:8">
       <c r="B42" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C42" t="s">
         <v>32</v>
@@ -8812,12 +8677,12 @@
         <v>4200</v>
       </c>
       <c r="H42" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="43" spans="2:8">
       <c r="B43" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C43" t="s">
         <v>32</v>
@@ -8835,12 +8700,12 @@
         <v>190</v>
       </c>
       <c r="H43" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="44" spans="2:8">
       <c r="B44" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C44" t="s">
         <v>36</v>
@@ -8863,7 +8728,7 @@
     </row>
     <row r="45" spans="2:8">
       <c r="B45" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C45" t="s">
         <v>36</v>
@@ -8881,12 +8746,12 @@
         <v>4000</v>
       </c>
       <c r="H45" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="46" spans="2:8">
       <c r="B46" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C46" t="s">
         <v>36</v>
@@ -8904,12 +8769,12 @@
         <v>170</v>
       </c>
       <c r="H46" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="47" spans="2:8">
       <c r="B47" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C47" t="s">
         <v>32</v>
@@ -8932,7 +8797,7 @@
     </row>
     <row r="48" spans="2:8">
       <c r="B48" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C48" t="s">
         <v>32</v>
@@ -8950,12 +8815,12 @@
         <v>4300</v>
       </c>
       <c r="H48" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="49" spans="2:8">
       <c r="B49" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C49" t="s">
         <v>32</v>
@@ -8973,12 +8838,12 @@
         <v>165</v>
       </c>
       <c r="H49" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="50" spans="2:8">
       <c r="B50" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C50" t="s">
         <v>27</v>
@@ -9001,7 +8866,7 @@
     </row>
     <row r="51" spans="2:8">
       <c r="B51" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C51" t="s">
         <v>27</v>
@@ -9019,12 +8884,12 @@
         <v>0.23</v>
       </c>
       <c r="H51" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="52" spans="2:8">
       <c r="B52" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C52" t="s">
         <v>27</v>
@@ -9042,12 +8907,12 @@
         <v>550</v>
       </c>
       <c r="H52" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="53" spans="2:8">
       <c r="B53" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C53" t="s">
         <v>27</v>
@@ -9065,12 +8930,12 @@
         <v>18</v>
       </c>
       <c r="H53" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="54" spans="2:8">
       <c r="B54" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C54" t="s">
         <v>27</v>
@@ -9088,12 +8953,12 @@
         <v>1.5</v>
       </c>
       <c r="H54" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="55" spans="2:8">
       <c r="B55" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C55" t="s">
         <v>32</v>
@@ -9116,7 +8981,7 @@
     </row>
     <row r="56" spans="2:8">
       <c r="B56" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C56" t="s">
         <v>32</v>
@@ -9134,12 +8999,12 @@
         <v>1300</v>
       </c>
       <c r="H56" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="57" spans="2:8">
       <c r="B57" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C57" t="s">
         <v>32</v>
@@ -9157,12 +9022,12 @@
         <v>45</v>
       </c>
       <c r="H57" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="58" spans="2:8">
       <c r="B58" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C58" t="s">
         <v>32</v>
@@ -9185,7 +9050,7 @@
     </row>
     <row r="59" spans="2:8">
       <c r="B59" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C59" t="s">
         <v>32</v>
@@ -9203,12 +9068,12 @@
         <v>1600</v>
       </c>
       <c r="H59" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="60" spans="2:8">
       <c r="B60" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C60" t="s">
         <v>32</v>
@@ -9226,12 +9091,12 @@
         <v>55</v>
       </c>
       <c r="H60" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="61" spans="2:8">
       <c r="B61" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C61" t="s">
         <v>32</v>
@@ -9254,7 +9119,7 @@
     </row>
     <row r="62" spans="2:8">
       <c r="B62" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C62" t="s">
         <v>32</v>
@@ -9272,12 +9137,12 @@
         <v>1900</v>
       </c>
       <c r="H62" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="63" spans="2:8">
       <c r="B63" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C63" t="s">
         <v>32</v>
@@ -9295,15 +9160,15 @@
         <v>70</v>
       </c>
       <c r="H63" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="64" spans="2:8">
       <c r="B64" t="s">
+        <v>334</v>
+      </c>
+      <c r="C64" t="s">
         <v>335</v>
-      </c>
-      <c r="C64" t="s">
-        <v>336</v>
       </c>
       <c r="D64" t="s">
         <v>19</v>
@@ -9323,10 +9188,10 @@
     </row>
     <row r="65" spans="2:8">
       <c r="B65" t="s">
+        <v>334</v>
+      </c>
+      <c r="C65" t="s">
         <v>335</v>
-      </c>
-      <c r="C65" t="s">
-        <v>336</v>
       </c>
       <c r="D65" t="s">
         <v>19</v>
@@ -9341,15 +9206,15 @@
         <v>0.43</v>
       </c>
       <c r="H65" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="66" spans="2:8">
       <c r="B66" t="s">
+        <v>334</v>
+      </c>
+      <c r="C66" t="s">
         <v>335</v>
-      </c>
-      <c r="C66" t="s">
-        <v>336</v>
       </c>
       <c r="D66" t="s">
         <v>19</v>
@@ -9364,15 +9229,15 @@
         <v>2200</v>
       </c>
       <c r="H66" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="67" spans="2:8">
       <c r="B67" t="s">
+        <v>334</v>
+      </c>
+      <c r="C67" t="s">
         <v>335</v>
-      </c>
-      <c r="C67" t="s">
-        <v>336</v>
       </c>
       <c r="D67" t="s">
         <v>19</v>
@@ -9387,15 +9252,15 @@
         <v>65</v>
       </c>
       <c r="H67" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="68" spans="2:8">
       <c r="B68" t="s">
+        <v>334</v>
+      </c>
+      <c r="C68" t="s">
         <v>335</v>
-      </c>
-      <c r="C68" t="s">
-        <v>336</v>
       </c>
       <c r="D68" t="s">
         <v>19</v>
@@ -9410,15 +9275,15 @@
         <v>3</v>
       </c>
       <c r="H68" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="69" spans="2:8">
       <c r="B69" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C69" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D69" t="s">
         <v>19</v>
@@ -9438,10 +9303,10 @@
     </row>
     <row r="70" spans="2:8">
       <c r="B70" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C70" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D70" t="s">
         <v>19</v>
@@ -9456,15 +9321,15 @@
         <v>0.35000000000000003</v>
       </c>
       <c r="H70" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="71" spans="2:8">
       <c r="B71" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C71" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D71" t="s">
         <v>19</v>
@@ -9479,15 +9344,15 @@
         <v>1470</v>
       </c>
       <c r="H71" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="72" spans="2:8">
       <c r="B72" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C72" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D72" t="s">
         <v>19</v>
@@ -9502,15 +9367,15 @@
         <v>38</v>
       </c>
       <c r="H72" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="73" spans="2:8">
       <c r="B73" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C73" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D73" t="s">
         <v>19</v>
@@ -9525,7 +9390,7 @@
         <v>1.5</v>
       </c>
       <c r="H73" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated ZWE model - 2025-09-16 23:50
</commit_message>
<xml_diff>
--- a/VerveStacks_ZWE/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ZWE/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZWE\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DF0F11A-84D9-4954-AD27-754541A75578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{24730C88-8D3B-431D-AC27-B9E7656164FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2573" yWindow="2573" windowWidth="21600" windowHeight="12682" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="12683" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc" sheetId="7" r:id="rId1"/>
@@ -6006,7 +6006,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{228CC0F7-74C7-4FFE-9724-9431B99186D6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69076E69-EDD6-4270-8BE7-A20CB42B3593}">
   <dimension ref="B9:M32"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6829,7 +6829,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF0BFFFF-66D7-4C40-A55E-3E9652F22240}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C6F860D-C90D-43F1-A342-B23A930A37D0}">
   <dimension ref="B9:M30"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7582,7 +7582,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B8F1400-49D2-4C36-8EB2-A47B5462D084}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50A0B681-69DE-481A-9B43-A0C9717185A5}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>